<commit_message>
feat: update manual curation logic, refine human verification conflict resolution, and implement cache-busting for data fetching
</commit_message>
<xml_diff>
--- a/final_antibiotics_curated_updated.xlsx
+++ b/final_antibiotics_curated_updated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ha-mim88\AntibioticGeneResistanceResearch\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ha-mim88\ARGResearchStage2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699E1998-7F13-4037-BCC6-5CE2D67A0F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C15F7F-BA17-4A77-BD8C-9B3F3CAD5B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41250" yWindow="6030" windowWidth="21480" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38970" yWindow="3750" windowWidth="21480" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="antibiotics" sheetId="1" r:id="rId1"/>
@@ -8027,11 +8027,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2242"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="4" max="4" width="34.08203125" customWidth="1"/>
-    <col min="5" max="5" width="38.58203125" customWidth="1"/>
-    <col min="6" max="6" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>